<commit_message>
Please enter the commit message for your changes. Lines starting with '#' will be ignored, and an empty message aborts the commit.
On branch main
Your branch is up to date with 'origin/main'.

Changes to be committed:
	modified:   Test/Mods/Mods/Mods_Archives.xlsx
	deleted:    Test/Mods/Mods/~$Mods_Archives.xlsx
</commit_message>
<xml_diff>
--- a/Test/Mods/Mods/Mods_Archives.xlsx
+++ b/Test/Mods/Mods/Mods_Archives.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LuLuLuOfficial\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Warehouse\Project\Program\_Projects\MineCraft Mod Vault Manager\Test\Mods\Mods\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC9DE92B-9150-4965-A808-4DBA39266530}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D36FCD68-F0D3-44D4-BE8D-F9EB3DECCDF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="2220" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-14505" yWindow="2340" windowWidth="14610" windowHeight="16305" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="163">
   <si>
     <t>Mod Name</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -35,10 +35,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Requirements [Mod ID]</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>carpet</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -423,26 +419,6 @@
   </si>
   <si>
     <t>I18nUpdateMod-3.6.0-all.jar</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>XPlus ContingameIME</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>xplus-contingameime</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>XPlusContingameIME-1.2.1-xplus-1.21.x-fabric.jar</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>[前置过多][Disabled]</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>…</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -521,10 +497,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>journeymap-fabric-1.21.4-6.0.0-beta.39.jar</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>essential-commands</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -702,6 +674,18 @@
   </si>
   <si>
     <t>Comments</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Depends</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[Disabled]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1051,7 +1035,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G50"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr defaultColWidth="25.77734375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="16384" width="25.77734375" style="1"/>
@@ -1059,22 +1043,22 @@
   <sheetData>
     <row r="1" spans="1:7" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>2</v>
+        <v>160</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>1</v>
@@ -1082,596 +1066,593 @@
     </row>
     <row r="2" spans="1:7" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>30</v>
       </c>
       <c r="D2" s="1"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>4</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="D4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="1" t="s">
-        <v>8</v>
-      </c>
       <c r="G4" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>12</v>
-      </c>
       <c r="D5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="1" t="s">
         <v>8</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="D6" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G6" s="1" t="s">
         <v>14</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="D7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G7" s="1" t="s">
         <v>17</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="D8" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G8" s="1" t="s">
         <v>20</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B9" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G9" s="1" t="s">
         <v>23</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B10" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="D10" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G10" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B11" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="G11" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B12" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G12" s="1" t="s">
         <v>51</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B13" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D13" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>38</v>
-      </c>
       <c r="G13" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B14" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="G14" s="1" t="s">
         <v>40</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B15" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C15" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="D15" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="G15" s="1" t="s">
         <v>43</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="G15" s="1" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B16" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="G16" s="1" t="s">
         <v>46</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B17" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C17" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C17" s="1" t="s">
-        <v>49</v>
-      </c>
       <c r="D17" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B18" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="G18" s="1" t="s">
         <v>55</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="G18" s="1" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B19" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="G19" s="1" t="s">
         <v>64</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="G19" s="1" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="G20" s="1" t="s">
         <v>67</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="G20" s="1" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B21" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="G21" s="1" t="s">
         <v>71</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="G21" s="1" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B22" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="G22" s="1" t="s">
         <v>74</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="G22" s="1" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B23" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="G23" s="1" t="s">
         <v>80</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="G23" s="1" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B24" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C24" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="C24" s="1" t="s">
+      <c r="G24" s="1" t="s">
         <v>58</v>
-      </c>
-      <c r="G24" s="1" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B25" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="G25" s="1" t="s">
         <v>61</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="G25" s="1" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B26" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="G26" s="1" t="s">
         <v>78</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="G26" s="1" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B27" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="G27" s="1" t="s">
         <v>84</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="G27" s="1" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B28" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="G28" s="1" t="s">
         <v>86</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="G28" s="1" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B29" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="G29" s="1" t="s">
         <v>90</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="G29" s="1" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B30" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="G30" s="1" t="s">
         <v>95</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="G30" s="1" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B31" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="G31" s="1" t="s">
         <v>92</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="G31" s="1" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B32" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="F32" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="G32" s="1" t="s">
         <v>98</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="F32" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="G32" s="1" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B33" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="G33" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="C33" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="F33" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="G33" s="1" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="34" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A34" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>105</v>
+        <v>109</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>112</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D35" s="1" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>117</v>
+        <v>162</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>123</v>
+        <v>133</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
     </row>
     <row r="38" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>140</v>
+        <v>130</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>138</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D39" s="1" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
       <c r="G39" s="1" t="s">
         <v>139</v>
@@ -1679,168 +1660,154 @@
     </row>
     <row r="40" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C40" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="G40" s="1" t="s">
         <v>143</v>
-      </c>
-      <c r="G40" s="1" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>149</v>
+        <v>119</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>148</v>
+        <v>118</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>147</v>
+        <v>112</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>150</v>
+        <v>120</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>126</v>
+        <v>146</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>127</v>
+        <v>145</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="D43" s="1" t="s">
-        <v>118</v>
+        <v>150</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>157</v>
+        <v>153</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>152</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>161</v>
+        <v>105</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="D45" s="1" t="s">
-        <v>159</v>
+        <v>104</v>
       </c>
       <c r="G45" s="1" t="s">
-        <v>158</v>
+        <v>106</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="G46" s="1" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>109</v>
+        <v>121</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>108</v>
+        <v>122</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
     </row>
     <row r="49" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="G49" s="1" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="50" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="B50" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="C50" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="G50" s="1" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
     </row>
   </sheetData>

</xml_diff>